<commit_message>
Cite the core queries by their new path in the competency question workbook
The "SPARQL Query File" column and one question text said queries/. They now say
ontology/queries/, so prov_augment.py no longer needs the mapping it carried since
the move. The regenerated record changes in that one question text.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/development/design/Competency Questions.xlsx
+++ b/development/design/Competency Questions.xlsx
@@ -542,7 +542,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>augmentation/queries/fc01_requirement_source.rq; queries/read_context_in_scope_for_goal.rq</t>
+          <t>augmentation/queries/fc01_requirement_source.rq; ontology/queries/read_context_in_scope_for_goal.rq</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>augmentation/queries/fc02_assured_system.rq; queries/read_context_in_scope_for_goal.rq</t>
+          <t>augmentation/queries/fc02_assured_system.rq; ontology/queries/read_context_in_scope_for_goal.rq</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>augmentation/queries/fc03_undeveloped_claims_for_system.rq; queries/read_context_in_scope_for_goal.rq; queries/read_undeveloped_elements.rq; queries/read_goals_without_support.rq</t>
+          <t>augmentation/queries/fc03_undeveloped_claims_for_system.rq; ontology/queries/read_context_in_scope_for_goal.rq; ontology/queries/read_undeveloped_elements.rq; ontology/queries/read_goals_without_support.rq</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>queries/read_goal_support_tree.rq</t>
+          <t>ontology/queries/read_goal_support_tree.rq</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>queries/read_goals_without_support.rq; queries/read_solutions_without_artefact.rq; queries/read_uninstantiated_elements.rq</t>
+          <t>ontology/queries/read_goals_without_support.rq; ontology/queries/read_solutions_without_artefact.rq; ontology/queries/read_uninstantiated_elements.rq</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>queries/read_evidence_supporting_goal.rq; queries/read_solutions_without_artefact.rq</t>
+          <t>ontology/queries/read_evidence_supporting_goal.rq; ontology/queries/read_solutions_without_artefact.rq</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>augmentation/queries/fc11_controls_ready_for_review.rq; queries/read_undeveloped_elements.rq</t>
+          <t>augmentation/queries/fc11_controls_ready_for_review.rq; ontology/queries/read_undeveloped_elements.rq</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>queries/read_element_status_flags.rq; queries/read_invalid_elements.rq</t>
+          <t>ontology/queries/read_element_status_flags.rq; ontology/queries/read_invalid_elements.rq</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>queries/read_challenges_and_their_targets.rq; queries/read_goals_affected_by_challenge.rq</t>
+          <t>ontology/queries/read_challenges_and_their_targets.rq; ontology/queries/read_goals_affected_by_challenge.rq</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>queries/read_element_status_flags.rq; queries/read_invalid_elements.rq</t>
+          <t>ontology/queries/read_element_status_flags.rq; ontology/queries/read_invalid_elements.rq</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>augmentation/queries/fc33_instantiated_elements.rq; queries/read_pattern_instantiations.rq</t>
+          <t>augmentation/queries/fc33_instantiated_elements.rq; ontology/queries/read_pattern_instantiations.rq</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>augmentation/queries/fc35_artefacts_to_change.rq; queries/read_goals_resting_on_artefact.rq</t>
+          <t>augmentation/queries/fc35_artefacts_to_change.rq; ontology/queries/read_goals_resting_on_artefact.rq</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>queries/read_assurance_case_inventory.rq</t>
+          <t>ontology/queries/read_assurance_case_inventory.rq</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>queries/read_assurance_claim_points.rq</t>
+          <t>ontology/queries/read_assurance_claim_points.rq</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>queries/read_away_elements.rq</t>
+          <t>ontology/queries/read_away_elements.rq</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>queries/read_case_summary_counts.rq</t>
+          <t>ontology/queries/read_case_summary_counts.rq</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>queries/read_claim_points_without_confidence_argument.rq</t>
+          <t>ontology/queries/read_claim_points_without_confidence_argument.rq</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>queries/read_duplicate_identifiers.rq</t>
+          <t>ontology/queries/read_duplicate_identifiers.rq</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>queries/read_element_by_identifier.rq</t>
+          <t>ontology/queries/read_element_by_identifier.rq</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>queries/read_elements_unreachable_from_top_goal.rq</t>
+          <t>ontology/queries/read_elements_unreachable_from_top_goal.rq</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>queries/read_module_dependencies.rq</t>
+          <t>ontology/queries/read_module_dependencies.rq</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>queries/read_public_elements_in_contract_modules.rq</t>
+          <t>ontology/queries/read_public_elements_in_contract_modules.rq</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>queries/read_relationship_decorators.rq</t>
+          <t>ontology/queries/read_relationship_decorators.rq</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>queries/read_stale_evidence.rq</t>
+          <t>ontology/queries/read_stale_evidence.rq</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>queries/read_support_cycles.rq</t>
+          <t>ontology/queries/read_support_cycles.rq</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>queries/read_top_goals.rq</t>
+          <t>ontology/queries/read_top_goals.rq</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>queries/create_assurance_case_skeleton.rq</t>
+          <t>ontology/queries/create_assurance_case_skeleton.rq</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>queries/create_challenge_to_element.rq</t>
+          <t>ontology/queries/create_challenge_to_element.rq</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>queries/create_context_for_goal.rq</t>
+          <t>ontology/queries/create_context_for_goal.rq</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>queries/create_goal_under_parent.rq</t>
+          <t>ontology/queries/create_goal_under_parent.rq</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>queries/create_solution_with_artefact.rq</t>
+          <t>ontology/queries/create_solution_with_artefact.rq</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>queries/create_solutions_for_unreferenced_artefacts.rq</t>
+          <t>ontology/queries/create_solutions_for_unreferenced_artefacts.rq</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>queries/create_strategy_between_goals.rq</t>
+          <t>ontology/queries/create_strategy_between_goals.rq</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>queries/update_element_statement.rq</t>
+          <t>ontology/queries/update_element_statement.rq</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>queries/update_mark_element_invalid.rq</t>
+          <t>ontology/queries/update_mark_element_invalid.rq</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>queries/update_retarget_solution_to_new_artefact.rq</t>
+          <t>ontology/queries/update_retarget_solution_to_new_artefact.rq</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>queries/delete_assurance_case.rq</t>
+          <t>ontology/queries/delete_assurance_case.rq</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>queries/delete_challenge_and_its_effects.rq</t>
+          <t>ontology/queries/delete_challenge_and_its_effects.rq</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>queries/delete_element_and_its_links.rq</t>
+          <t>ontology/queries/delete_element_and_its_links.rq</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2289,12 +2289,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>How are the conclusions written by queries/rules/ cleared before re-running them?</t>
+          <t>How are the conclusions written by ontology/queries/rules/ cleared before re-running them?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>queries/delete_materialised_inferences.rq</t>
+          <t>ontology/queries/delete_materialised_inferences.rq</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>queries/delete_support_link.rq</t>
+          <t>ontology/queries/delete_support_link.rq</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>queries/delete_unreferenced_artefacts.rq</t>
+          <t>ontology/queries/delete_unreferenced_artefacts.rq</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">

</xml_diff>